<commit_message>
Add published LLM travel behavior paper
</commit_message>
<xml_diff>
--- a/documents/papers.xlsx
+++ b/documents/papers.xlsx
@@ -1008,11 +1008,11 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Baichuan Mo, Hanyong Xu, Dingyi Zhuang, Ruoyun Ma, Xiaotong Guo, Jinhua Zhao</t>
+          <t>Baichuan Mo, Hanyong Xu, Ruoyun Ma, Jung-Hoon Cho, Dingyi Zhuang, Xiaotong Guo, Jinhua Zhao</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1022,21 +1022,32 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
+          <t>https://doi.org/10.1016/j.trip.2026.102124</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3.8</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
-        </is>
-      </c>
-      <c r="K11" s="1" t="n">
-        <v>2312.00819</v>
+          <t>Transportation Research Interdisciplinary Perspectives</t>
+        </is>
+      </c>
+      <c r="K11" s="1" t="inlineStr">
+        <is>
+          <t>38, 102124</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Update CV publication details
</commit_message>
<xml_diff>
--- a/documents/papers.xlsx
+++ b/documents/papers.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R385af7c3d1234111"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1a5613f702d542d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1283,10 +1283,8 @@
           <x:t xml:space="preserve">Transportation Science</x:t>
         </x:is>
       </x:c>
-      <x:c r="K18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Accepted</x:t>
-        </x:is>
+      <x:c r="K18" t="str">
+        <x:v>59 (6), 1235-1258</x:v>
       </x:c>
       <x:c r="L18" t="n">
         <x:v>1</x:v>
@@ -2375,10 +2373,8 @@
           <x:t xml:space="preserve">Nature Sustainability</x:t>
         </x:is>
       </x:c>
-      <x:c r="K41" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Accepted</x:t>
-        </x:is>
+      <x:c r="K41" t="str">
+        <x:v>8, 1259-1269</x:v>
       </x:c>
       <x:c r="L41" t="n">
         <x:v>1</x:v>
@@ -2668,18 +2664,18 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="R8a70640037154634"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R8b6da580ee224c0e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="R38b9e3058d62400d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="R7734bcb81a534c4c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R95bf6b0c674d4788"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="Rc8e3d3c4e21041ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="Re37076c9b18d41cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R47983b41dd2c4c4e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="R42f7df090667409b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="R804c963894cd4fdc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="Re0a29c3e5f824751"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="R86a4fe2e66554f25"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="R145c0cef26d5411a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R28a7f98f78c349da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="Rd54241187a224789"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="Ra77dd8ada5804ea6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R7032ab06517e4848"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="Rc1c22a971a4146f4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="R0d977db71f384477"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R6c86e7b30b3c4ccb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="R4ed8b85cea024458"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="R0437be5eb9784153"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="R4cd305ded44a455f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="Rfdd78296e3cb4eac"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add publication issue numbers across site and CV
</commit_message>
<xml_diff>
--- a/documents/papers.xlsx
+++ b/documents/papers.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1a5613f702d542d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5173a10e1ca540d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2374,7 +2374,7 @@
         </x:is>
       </x:c>
       <x:c r="K41" t="str">
-        <x:v>8, 1259-1269</x:v>
+        <x:v>8 (11), 1259-1269</x:v>
       </x:c>
       <x:c r="L41" t="n">
         <x:v>1</x:v>
@@ -2507,10 +2507,8 @@
           <x:t xml:space="preserve">Communications in Transportation Research</x:t>
         </x:is>
       </x:c>
-      <x:c r="K44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">6, 9640014</x:t>
-        </x:is>
+      <x:c r="K44" t="str">
+        <x:v>6 (1), 9640014</x:v>
       </x:c>
       <x:c r="L44" t="n">
         <x:v>0</x:v>
@@ -2664,18 +2662,18 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="R145c0cef26d5411a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R28a7f98f78c349da"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="Rd54241187a224789"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="Ra77dd8ada5804ea6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R7032ab06517e4848"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="Rc1c22a971a4146f4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="R0d977db71f384477"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R6c86e7b30b3c4ccb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="R4ed8b85cea024458"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="R0437be5eb9784153"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="R4cd305ded44a455f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="Rfdd78296e3cb4eac"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="Rcb1021ae9bec4622"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R85234c05548e47a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="R11710b48c88f40c2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="R2936c6fbc6774b73"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="Rf09df989dcb74dea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="R1cf8aae45cdb434e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="Rd80e02ec78e84e13"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R801926796324490b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="R9849408f478148ff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="Rb0746f3e9a094a33"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="R1f1a45322dfb443f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="R169fef35d5364cf4"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add book chapter and update award records
</commit_message>
<xml_diff>
--- a/documents/papers.xlsx
+++ b/documents/papers.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5173a10e1ca540d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc8f8869b34974483"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2643,18 +2643,34 @@
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47"/>
-      <x:c r="B47"/>
-      <x:c r="C47"/>
+      <x:c r="A47" t="str">
+        <x:v>User-centric transit data analytics for inference, prediction, and optimization</x:v>
+      </x:c>
+      <x:c r="B47" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>Zhenliang Ma, Haris N. Koutsopoulos, Baichuan Mo, Jinhua Zhao</x:v>
+      </x:c>
       <x:c r="D47"/>
       <x:c r="E47"/>
-      <x:c r="F47"/>
+      <x:c r="F47" t="str">
+        <x:v>https://doi.org/10.1016/B978-0-443-26789-5.00018-3</x:v>
+      </x:c>
       <x:c r="G47"/>
       <x:c r="H47"/>
-      <x:c r="I47"/>
-      <x:c r="J47"/>
-      <x:c r="K47"/>
-      <x:c r="L47"/>
+      <x:c r="I47" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>Mobility Patterns, Big Data and Transport Analytics (2nd ed.)</x:v>
+      </x:c>
+      <x:c r="K47" t="str">
+        <x:v>421-461</x:v>
+      </x:c>
+      <x:c r="L47" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="M47"/>
       <x:c r="N47"/>
       <x:c r="O47"/>
@@ -2662,18 +2678,18 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="Rcb1021ae9bec4622"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R85234c05548e47a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="R11710b48c88f40c2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="R2936c6fbc6774b73"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="Rf09df989dcb74dea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="R1cf8aae45cdb434e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="Rd80e02ec78e84e13"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R801926796324490b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="R9849408f478148ff"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="Rb0746f3e9a094a33"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="R1f1a45322dfb443f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="R169fef35d5364cf4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="R7dde7a2e14d249fc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R8dd7c82cd9d54041"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="Rc8a1034a607744ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="Re7b69e4f3c394f16"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R071d84a415f04b64"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="Rcf6a1fe7a783486b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="R5fe68630a3414352"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R0948d6c07d6445db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="Raccb8d93fd954d05"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="Rff08020149e74e81"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="R48c51bf1067a481d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="Re9ee0b5534ec431c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>